<commit_message>
#31 0R resistor added in BOM
</commit_message>
<xml_diff>
--- a/Design Files/LoRaWAN-Module-v2.0/BOM/Client_BOM_LoRaWAN-Module-v2.0.xlsx
+++ b/Design Files/LoRaWAN-Module-v2.0/BOM/Client_BOM_LoRaWAN-Module-v2.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\chrisbyrd-esp32iotproduct\Design Files\LoRaWAN-Module-v2.0\LoRaWAN-Module-v2.0\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\chrisbyrd-esp32iotproduct\Design Files\LoRaWAN-Module-v2.0\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -69,9 +69,6 @@
     <t>J2</t>
   </si>
   <si>
-    <t>R1, R2, R3, R4</t>
-  </si>
-  <si>
     <t>U1</t>
   </si>
   <si>
@@ -90,9 +87,6 @@
     <t>1 Inner bore SMA Board Edge Bend -55℃~+155℃ 50Ω Plugin RF Connectors / Coaxial Connectors ROHS</t>
   </si>
   <si>
-    <t>RES SMD 10K OHM 1% 1/20W 0201</t>
-  </si>
-  <si>
     <t>SMD,16x16mm LoRa Modules ROHS</t>
   </si>
   <si>
@@ -108,9 +102,6 @@
     <t>HJ-SMA508_</t>
   </si>
   <si>
-    <t>Res-0201</t>
-  </si>
-  <si>
     <t>SX1276S8S+T-X1</t>
   </si>
   <si>
@@ -126,9 +117,6 @@
     <t>HJ-SMA508</t>
   </si>
   <si>
-    <t>RC0201FR-0710KL</t>
-  </si>
-  <si>
     <t>Manufacturer</t>
   </si>
   <si>
@@ -147,9 +135,6 @@
     <t>0.1uF</t>
   </si>
   <si>
-    <t>10K</t>
-  </si>
-  <si>
     <t>Quantity</t>
   </si>
   <si>
@@ -193,6 +178,21 @@
   </si>
   <si>
     <t>LoRaWAN-Module-v2.0.</t>
+  </si>
+  <si>
+    <t>R1, R2</t>
+  </si>
+  <si>
+    <t>RES SMD 0R, 1%, 0.1W, 0603</t>
+  </si>
+  <si>
+    <t>Res-0603</t>
+  </si>
+  <si>
+    <t>RC0603FR-070RL</t>
+  </si>
+  <si>
+    <t>0R</t>
   </si>
 </sst>
 </file>
@@ -737,6 +737,39 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="3" borderId="14" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -745,39 +778,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="3" borderId="14" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1151,13 +1151,13 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="53"/>
-      <c r="K1" s="53"/>
-      <c r="L1" s="53"/>
-      <c r="M1" s="53"/>
-      <c r="N1" s="53"/>
-      <c r="O1" s="53"/>
-      <c r="P1" s="53"/>
+      <c r="J1" s="64"/>
+      <c r="K1" s="64"/>
+      <c r="L1" s="64"/>
+      <c r="M1" s="64"/>
+      <c r="N1" s="64"/>
+      <c r="O1" s="64"/>
+      <c r="P1" s="64"/>
     </row>
     <row r="2" spans="1:16" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1168,7 +1168,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="49" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
@@ -1190,7 +1190,7 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="50" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
@@ -1201,7 +1201,7 @@
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
-      <c r="P3" s="54"/>
+      <c r="P3" s="65"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="51" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
@@ -1223,7 +1223,7 @@
       <c r="M4" s="5"/>
       <c r="N4" s="5"/>
       <c r="O4" s="5"/>
-      <c r="P4" s="55"/>
+      <c r="P4" s="66"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1245,7 +1245,7 @@
       <c r="M5" s="5"/>
       <c r="N5" s="5"/>
       <c r="O5" s="5"/>
-      <c r="P5" s="55"/>
+      <c r="P5" s="66"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1263,7 +1263,7 @@
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
       <c r="O6" s="5"/>
-      <c r="P6" s="55"/>
+      <c r="P6" s="66"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1281,7 +1281,7 @@
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
-      <c r="P7" s="55"/>
+      <c r="P7" s="66"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1299,7 +1299,7 @@
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
       <c r="O8" s="7"/>
-      <c r="P8" s="55"/>
+      <c r="P8" s="66"/>
     </row>
     <row r="9" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1313,40 +1313,40 @@
         <v>11</v>
       </c>
       <c r="E9" s="30" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="I9" s="29" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="J9" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="K9" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="L9" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="M9" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="N9" s="29" t="s">
+        <v>46</v>
+      </c>
+      <c r="O9" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="K9" s="29" t="s">
-        <v>43</v>
-      </c>
-      <c r="L9" s="29" t="s">
+      <c r="P9" s="29" t="s">
         <v>48</v>
-      </c>
-      <c r="M9" s="29" t="s">
-        <v>50</v>
-      </c>
-      <c r="N9" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="O9" s="29" t="s">
-        <v>52</v>
-      </c>
-      <c r="P9" s="29" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1355,27 +1355,27 @@
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="56" t="s">
+      <c r="C10" s="53" t="s">
         <v>7</v>
       </c>
       <c r="D10" s="36" t="s">
         <v>12</v>
       </c>
       <c r="E10" s="36" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G10" s="36" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H10" s="36"/>
       <c r="I10" s="36" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="J10" s="36" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="K10" s="36">
         <v>1</v>
@@ -1384,13 +1384,13 @@
         <f>K10*5</f>
         <v>5</v>
       </c>
-      <c r="M10" s="59" t="s">
-        <v>54</v>
-      </c>
-      <c r="N10" s="60">
+      <c r="M10" s="56" t="s">
+        <v>49</v>
+      </c>
+      <c r="N10" s="57">
         <v>0.1</v>
       </c>
-      <c r="O10" s="61">
+      <c r="O10" s="58">
         <f>N10*L10</f>
         <v>0.5</v>
       </c>
@@ -1402,27 +1402,27 @@
         <f t="shared" ref="B11:B15" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="56" t="s">
+      <c r="C11" s="53" t="s">
         <v>7</v>
       </c>
       <c r="D11" s="37" t="s">
         <v>13</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>26</v>
-      </c>
-      <c r="G11" s="66" t="s">
-        <v>33</v>
+        <v>24</v>
+      </c>
+      <c r="G11" s="63" t="s">
+        <v>30</v>
       </c>
       <c r="H11" s="37"/>
       <c r="I11" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="J11" s="37" t="s">
         <v>37</v>
-      </c>
-      <c r="J11" s="37" t="s">
-        <v>41</v>
       </c>
       <c r="K11" s="37">
         <v>1</v>
@@ -1431,13 +1431,13 @@
         <f t="shared" ref="L11" si="1">K11*5</f>
         <v>5</v>
       </c>
-      <c r="M11" s="59" t="s">
-        <v>54</v>
-      </c>
-      <c r="N11" s="60">
+      <c r="M11" s="56" t="s">
+        <v>49</v>
+      </c>
+      <c r="N11" s="57">
         <v>0.1</v>
       </c>
-      <c r="O11" s="60">
+      <c r="O11" s="57">
         <f t="shared" ref="O11" si="2">N11*L11</f>
         <v>0.5</v>
       </c>
@@ -1449,41 +1449,41 @@
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="58" t="s">
-        <v>44</v>
-      </c>
-      <c r="D12" s="57" t="s">
+      <c r="C12" s="55" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" s="54" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="57" t="s">
-        <v>21</v>
-      </c>
-      <c r="F12" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="G12" s="57" t="s">
-        <v>45</v>
+      <c r="E12" s="54" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12" s="54" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="54" t="s">
+        <v>40</v>
       </c>
       <c r="H12" s="36"/>
-      <c r="I12" s="57" t="s">
-        <v>45</v>
-      </c>
-      <c r="J12" s="57" t="s">
-        <v>45</v>
-      </c>
-      <c r="K12" s="57">
+      <c r="I12" s="54" t="s">
+        <v>40</v>
+      </c>
+      <c r="J12" s="54" t="s">
+        <v>40</v>
+      </c>
+      <c r="K12" s="54">
         <v>1</v>
       </c>
-      <c r="L12" s="57">
+      <c r="L12" s="54">
         <f>K12*5</f>
         <v>5</v>
       </c>
-      <c r="M12" s="57"/>
-      <c r="N12" s="62" t="s">
-        <v>45</v>
-      </c>
-      <c r="O12" s="62" t="s">
-        <v>45</v>
+      <c r="M12" s="54"/>
+      <c r="N12" s="59" t="s">
+        <v>40</v>
+      </c>
+      <c r="O12" s="59" t="s">
+        <v>40</v>
       </c>
       <c r="P12" s="36"/>
     </row>
@@ -1493,27 +1493,27 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="56" t="s">
+      <c r="C13" s="53" t="s">
         <v>8</v>
       </c>
       <c r="D13" s="37" t="s">
         <v>15</v>
       </c>
       <c r="E13" s="37" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F13" s="37" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G13" s="37" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="H13" s="37"/>
       <c r="I13" s="37" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="J13" s="37" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="K13" s="37">
         <v>1</v>
@@ -1522,11 +1522,11 @@
         <f t="shared" ref="L13" si="3">K13*5</f>
         <v>5</v>
       </c>
-      <c r="M13" s="63" t="s">
-        <v>55</v>
-      </c>
-      <c r="N13" s="60"/>
-      <c r="O13" s="60">
+      <c r="M13" s="60" t="s">
+        <v>50</v>
+      </c>
+      <c r="N13" s="57"/>
+      <c r="O13" s="57">
         <f t="shared" ref="O13" si="4">N13*L13</f>
         <v>0</v>
       </c>
@@ -1538,27 +1538,27 @@
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
-      <c r="C14" s="58" t="s">
+      <c r="C14" s="55" t="s">
         <v>9</v>
       </c>
       <c r="D14" s="36" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="E14" s="36" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="G14" s="36" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="H14" s="36"/>
       <c r="I14" s="36" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="J14" s="36" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="K14" s="36">
         <v>4</v>
@@ -1567,13 +1567,13 @@
         <f>K14*5</f>
         <v>20</v>
       </c>
-      <c r="M14" s="63" t="s">
-        <v>54</v>
-      </c>
-      <c r="N14" s="61">
+      <c r="M14" s="60" t="s">
+        <v>49</v>
+      </c>
+      <c r="N14" s="58">
         <v>0.1</v>
       </c>
-      <c r="O14" s="61">
+      <c r="O14" s="58">
         <f>N14*L14</f>
         <v>2</v>
       </c>
@@ -1585,27 +1585,27 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="56" t="s">
+      <c r="C15" s="53" t="s">
         <v>10</v>
       </c>
       <c r="D15" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E15" s="37" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F15" s="37" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="G15" s="37" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H15" s="37"/>
       <c r="I15" s="37" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="J15" s="37" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="K15" s="37">
         <v>1</v>
@@ -1614,11 +1614,11 @@
         <f t="shared" ref="L15" si="5">K15*5</f>
         <v>5</v>
       </c>
-      <c r="M15" s="59" t="s">
-        <v>55</v>
-      </c>
-      <c r="N15" s="60"/>
-      <c r="O15" s="60">
+      <c r="M15" s="56" t="s">
+        <v>50</v>
+      </c>
+      <c r="N15" s="57"/>
+      <c r="O15" s="57">
         <f t="shared" ref="O15" si="6">N15*L15</f>
         <v>0</v>
       </c>
@@ -1639,7 +1639,7 @@
       <c r="L16" s="35"/>
       <c r="M16" s="35"/>
       <c r="N16" s="35"/>
-      <c r="O16" s="64">
+      <c r="O16" s="61">
         <f>SUM(O10:O15)</f>
         <v>3</v>
       </c>
@@ -1660,7 +1660,7 @@
       <c r="L17" s="9"/>
       <c r="M17" s="9"/>
       <c r="N17" s="9"/>
-      <c r="O17" s="65">
+      <c r="O17" s="62">
         <f>O16/5</f>
         <v>0.6</v>
       </c>

</xml_diff>

<commit_message>
#31 Antenna Added in Peripheral
</commit_message>
<xml_diff>
--- a/Design Files/LoRaWAN-Module-v2.0/BOM/Client_BOM_LoRaWAN-Module-v2.0.xlsx
+++ b/Design Files/LoRaWAN-Module-v2.0/BOM/Client_BOM_LoRaWAN-Module-v2.0.xlsx
@@ -12,14 +12,14 @@
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="61">
   <si>
     <t>Component list</t>
   </si>
@@ -193,6 +193,15 @@
   </si>
   <si>
     <t>0R</t>
+  </si>
+  <si>
+    <t>Peripheral</t>
+  </si>
+  <si>
+    <t>4 Rubber rod antenna 2.4GHz - Antennas ROHS</t>
+  </si>
+  <si>
+    <t>RF2111027</t>
   </si>
 </sst>
 </file>
@@ -598,7 +607,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -778,6 +787,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1121,7 +1136,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -1370,7 +1385,9 @@
       <c r="G10" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="H10" s="36"/>
+      <c r="H10" s="36" t="s">
+        <v>40</v>
+      </c>
       <c r="I10" s="36" t="s">
         <v>33</v>
       </c>
@@ -1399,7 +1416,7 @@
     <row r="11" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="48">
-        <f t="shared" ref="B11:B15" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B16" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="53" t="s">
@@ -1417,7 +1434,9 @@
       <c r="G11" s="63" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="37"/>
+      <c r="H11" s="37" t="s">
+        <v>40</v>
+      </c>
       <c r="I11" s="37" t="s">
         <v>33</v>
       </c>
@@ -1464,7 +1483,9 @@
       <c r="G12" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="H12" s="36"/>
+      <c r="H12" s="36" t="s">
+        <v>40</v>
+      </c>
       <c r="I12" s="54" t="s">
         <v>40</v>
       </c>
@@ -1508,7 +1529,9 @@
       <c r="G13" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="H13" s="37"/>
+      <c r="H13" s="37" t="s">
+        <v>40</v>
+      </c>
       <c r="I13" s="37" t="s">
         <v>34</v>
       </c>
@@ -1553,7 +1576,9 @@
       <c r="G14" s="36" t="s">
         <v>56</v>
       </c>
-      <c r="H14" s="36"/>
+      <c r="H14" s="36" t="s">
+        <v>40</v>
+      </c>
       <c r="I14" s="36" t="s">
         <v>33</v>
       </c>
@@ -1579,7 +1604,7 @@
       </c>
       <c r="P14" s="36"/>
     </row>
-    <row r="15" spans="1:16" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="48">
         <f t="shared" si="0"/>
@@ -1600,7 +1625,9 @@
       <c r="G15" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="H15" s="37"/>
+      <c r="H15" s="37" t="s">
+        <v>40</v>
+      </c>
       <c r="I15" s="37" t="s">
         <v>35</v>
       </c>
@@ -1611,60 +1638,105 @@
         <v>1</v>
       </c>
       <c r="L15" s="37">
-        <f t="shared" ref="L15" si="5">K15*5</f>
+        <f t="shared" ref="L15:L16" si="5">K15*5</f>
         <v>5</v>
       </c>
       <c r="M15" s="56" t="s">
         <v>50</v>
       </c>
       <c r="N15" s="57"/>
-      <c r="O15" s="57">
-        <f t="shared" ref="O15" si="6">N15*L15</f>
-        <v>0</v>
+      <c r="O15" s="57" t="s">
+        <v>40</v>
       </c>
       <c r="P15" s="37"/>
     </row>
-    <row r="16" spans="1:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="31"/>
-      <c r="C16" s="46"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="34"/>
-      <c r="G16" s="35"/>
-      <c r="H16" s="35"/>
-      <c r="I16" s="34"/>
-      <c r="J16" s="35"/>
-      <c r="K16" s="35"/>
-      <c r="L16" s="35"/>
-      <c r="M16" s="35"/>
-      <c r="N16" s="35"/>
-      <c r="O16" s="61">
-        <f>SUM(O10:O15)</f>
-        <v>3</v>
-      </c>
-      <c r="P16" s="39"/>
+      <c r="B16" s="48">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="C16" s="53" t="s">
+        <v>58</v>
+      </c>
+      <c r="D16" s="37" t="s">
+        <v>40</v>
+      </c>
+      <c r="E16" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="F16" s="37" t="s">
+        <v>40</v>
+      </c>
+      <c r="G16" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="H16" s="67" t="s">
+        <v>40</v>
+      </c>
+      <c r="I16" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="J16" s="37" t="s">
+        <v>40</v>
+      </c>
+      <c r="K16" s="67">
+        <v>1</v>
+      </c>
+      <c r="L16" s="37">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="M16" s="60" t="s">
+        <v>50</v>
+      </c>
+      <c r="N16" s="57"/>
+      <c r="O16" s="57" t="s">
+        <v>40</v>
+      </c>
+      <c r="P16" s="68"/>
     </row>
     <row r="17" spans="1:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
-      <c r="B17" s="24"/>
-      <c r="C17" s="47"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
-      <c r="K17" s="9"/>
-      <c r="L17" s="9"/>
-      <c r="M17" s="9"/>
-      <c r="N17" s="9"/>
-      <c r="O17" s="62">
-        <f>O16/5</f>
+      <c r="B17" s="31"/>
+      <c r="C17" s="46"/>
+      <c r="D17" s="32"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="34"/>
+      <c r="G17" s="35"/>
+      <c r="H17" s="35"/>
+      <c r="I17" s="34"/>
+      <c r="J17" s="35"/>
+      <c r="K17" s="35"/>
+      <c r="L17" s="35"/>
+      <c r="M17" s="35"/>
+      <c r="N17" s="35"/>
+      <c r="O17" s="61">
+        <f>SUM(O10:O16)</f>
+        <v>3</v>
+      </c>
+      <c r="P17" s="39"/>
+    </row>
+    <row r="18" spans="1:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="1"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="47"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="9"/>
+      <c r="K18" s="9"/>
+      <c r="L18" s="9"/>
+      <c r="M18" s="9"/>
+      <c r="N18" s="9"/>
+      <c r="O18" s="62">
+        <f>O17/5</f>
         <v>0.6</v>
       </c>
-      <c r="P17" s="40"/>
+      <c r="P18" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
#31 Antenna Change in BOM.
</commit_message>
<xml_diff>
--- a/Design Files/LoRaWAN-Module-v2.0/BOM/Client_BOM_LoRaWAN-Module-v2.0.xlsx
+++ b/Design Files/LoRaWAN-Module-v2.0/BOM/Client_BOM_LoRaWAN-Module-v2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="62">
   <si>
     <t>Component list</t>
   </si>
@@ -198,10 +198,13 @@
     <t>Peripheral</t>
   </si>
   <si>
-    <t>4 Rubber rod antenna 2.4GHz - Antennas ROHS</t>
-  </si>
-  <si>
-    <t>RF2111027</t>
+    <t>1.8 3dBi Vertical 50W - Antennas ROHS</t>
+  </si>
+  <si>
+    <t>BW868JWX105-10KJ</t>
+  </si>
+  <si>
+    <t>BAT WIRELESS</t>
   </si>
 </sst>
 </file>
@@ -779,6 +782,12 @@
     <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -787,12 +796,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1166,13 +1169,13 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="64"/>
-      <c r="O1" s="64"/>
-      <c r="P1" s="64"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="66"/>
+      <c r="L1" s="66"/>
+      <c r="M1" s="66"/>
+      <c r="N1" s="66"/>
+      <c r="O1" s="66"/>
+      <c r="P1" s="66"/>
     </row>
     <row r="2" spans="1:16" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1216,7 +1219,7 @@
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
-      <c r="P3" s="65"/>
+      <c r="P3" s="67"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1238,7 +1241,7 @@
       <c r="M4" s="5"/>
       <c r="N4" s="5"/>
       <c r="O4" s="5"/>
-      <c r="P4" s="66"/>
+      <c r="P4" s="68"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1260,7 +1263,7 @@
       <c r="M5" s="5"/>
       <c r="N5" s="5"/>
       <c r="O5" s="5"/>
-      <c r="P5" s="66"/>
+      <c r="P5" s="68"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1278,7 +1281,7 @@
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
       <c r="O6" s="5"/>
-      <c r="P6" s="66"/>
+      <c r="P6" s="68"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1296,7 +1299,7 @@
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
-      <c r="P7" s="66"/>
+      <c r="P7" s="68"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1314,7 +1317,7 @@
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
       <c r="O8" s="7"/>
-      <c r="P8" s="66"/>
+      <c r="P8" s="68"/>
     </row>
     <row r="9" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1671,16 +1674,16 @@
       <c r="G16" s="37" t="s">
         <v>60</v>
       </c>
-      <c r="H16" s="67" t="s">
+      <c r="H16" s="64" t="s">
         <v>40</v>
       </c>
       <c r="I16" s="37" t="s">
-        <v>34</v>
+        <v>61</v>
       </c>
       <c r="J16" s="37" t="s">
         <v>40</v>
       </c>
-      <c r="K16" s="67">
+      <c r="K16" s="64">
         <v>1</v>
       </c>
       <c r="L16" s="37">
@@ -1694,7 +1697,7 @@
       <c r="O16" s="57" t="s">
         <v>40</v>
       </c>
-      <c r="P16" s="68"/>
+      <c r="P16" s="65"/>
     </row>
     <row r="17" spans="1:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>

</xml_diff>